<commit_message>
chore(import): limpiar metadatos personales de la muestra de Excel real
Se eliminan autor, último modificador y compañía de docProps con el
Inspector de documentos de Excel. Las celdas no cambian: el lector y la
integración de imports siguen en verde con el archivo.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/excel-real/excel-real-sample.xlsx
+++ b/data/samples/excel-real/excel-real-sample.xlsx
@@ -2,13 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\recon-tool-2\data\samples\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6995EAB-4CC4-4D22-8647-2D895E7E24B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22BA686B-88DD-499E-BE2E-3415538F13E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{404F2FA8-9B8A-4AC6-A258-4D88D8C7F8AF}"/>
   </bookViews>

</xml_diff>